<commit_message>
Uji bahwa baris lanjutan boleh mengosongkan kolom keterangan donatur
Berkas contoh dengan nama kosong di baris ke-2 dan seterusnya terbaca sebagai
kelalaian pengisian, padahal importer memang hanya membaca kolom keterangan dari
baris pertama kemunculan sebuah kode. Tanpa uji, kekhawatiran itu wajar dan tidak
bisa dijawab.

Dua uji ditambahkan: baris lanjutan yang kosong tetap menghasilkan satu donatur
dengan 17 mushaf (bukan berhenti di baris pertama), dan keterangan yang justru
diisi di baris lanjutan tetap dihormati.

Berkas contohnya diperbarui: seluruh kolom donatur kini diisi penuh di setiap
baris, supaya tidak ada sel kosong yang terbaca sebagai kelewat diisi.
</commit_message>
<xml_diff>
--- a/tests/fixtures/data-dummy-donatur-10.xlsx
+++ b/tests/fixtures/data-dummy-donatur-10.xlsx
@@ -709,10 +709,26 @@
           <t>DMY003</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Hj. Nurhayati</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>6281234500003</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>nurhayati@contoh.id</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Pagesangan Asri No. 21, Kel. Pagesangan, Kec. Jambangan, Surabaya 60233</t>
+        </is>
+      </c>
       <c r="F5" s="5" t="n">
         <v>5</v>
       </c>
@@ -722,7 +738,11 @@
       <c r="H5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="inlineStr">
         <is>
@@ -803,10 +823,26 @@
           <t>DMY004</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Bapak Sukarno Wibowo</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>081234500004</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>sukarno.wibowo@contoh.id</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Gedongkiwo MJ I/123, Kel. Gedongkiwo, Kec. Mantrijeron, Yogyakarta 55142</t>
+        </is>
+      </c>
       <c r="F7" s="5" t="n">
         <v>3</v>
       </c>
@@ -816,7 +852,11 @@
       <c r="H7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="5" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>15/01/2026</t>
+        </is>
+      </c>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="inlineStr">
         <is>
@@ -840,10 +880,26 @@
           <t>DMY004</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Bapak Sukarno Wibowo</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>081234500004</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>sukarno.wibowo@contoh.id</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Gedongkiwo MJ I/123, Kel. Gedongkiwo, Kec. Mantrijeron, Yogyakarta 55142</t>
+        </is>
+      </c>
       <c r="F8" s="5" t="n">
         <v>0</v>
       </c>
@@ -853,7 +909,11 @@
       <c r="H8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>15/01/2026</t>
+        </is>
+      </c>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="inlineStr">
         <is>
@@ -934,7 +994,11 @@
           <t>081234500006</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>rizki.pratama@contoh.id</t>
+        </is>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Jl. Bontorannu No. 8, Kel. Bontorannu, Kec. Mariso, Makassar 90121</t>
@@ -975,10 +1039,26 @@
           <t>DMY006</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Muhammad Rizki Pratama</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>081234500006</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>rizki.pratama@contoh.id</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Bontorannu No. 8, Kel. Bontorannu, Kec. Mariso, Makassar 90121</t>
+        </is>
+      </c>
       <c r="F11" s="5" t="n">
         <v>1</v>
       </c>
@@ -988,7 +1068,9 @@
       <c r="H11" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I11" s="5" t="n"/>
+      <c r="I11" s="6" t="n">
+        <v>46033</v>
+      </c>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="inlineStr">
         <is>
@@ -1012,10 +1094,26 @@
           <t>DMY006</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Muhammad Rizki Pratama</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>081234500006</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>rizki.pratama@contoh.id</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Bontorannu No. 8, Kel. Bontorannu, Kec. Mariso, Makassar 90121</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="n">
         <v>1</v>
       </c>
@@ -1025,7 +1123,9 @@
       <c r="H12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="5" t="n"/>
+      <c r="I12" s="6" t="n">
+        <v>46033</v>
+      </c>
       <c r="J12" s="5" t="n"/>
       <c r="K12" s="5" t="inlineStr">
         <is>
@@ -1049,10 +1149,26 @@
           <t>DMY006</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Muhammad Rizki Pratama</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>081234500006</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>rizki.pratama@contoh.id</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Bontorannu No. 8, Kel. Bontorannu, Kec. Mariso, Makassar 90121</t>
+        </is>
+      </c>
       <c r="F13" s="5" t="n">
         <v>1</v>
       </c>
@@ -1062,7 +1178,9 @@
       <c r="H13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I13" s="5" t="n"/>
+      <c r="I13" s="6" t="n">
+        <v>46033</v>
+      </c>
       <c r="J13" s="5" t="n"/>
       <c r="K13" s="5" t="inlineStr">
         <is>
@@ -1086,10 +1204,26 @@
           <t>DMY006</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Muhammad Rizki Pratama</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>081234500006</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>rizki.pratama@contoh.id</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Bontorannu No. 8, Kel. Bontorannu, Kec. Mariso, Makassar 90121</t>
+        </is>
+      </c>
       <c r="F14" s="5" t="n">
         <v>1</v>
       </c>
@@ -1099,7 +1233,9 @@
       <c r="H14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="5" t="n"/>
+      <c r="I14" s="6" t="n">
+        <v>46033</v>
+      </c>
       <c r="J14" s="5" t="n"/>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -1133,7 +1269,11 @@
           <t>081234500007</t>
         </is>
       </c>
-      <c r="D15" s="5" t="n"/>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>dewi.anggraini@contoh.id</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Jl. Cangkiran Raya No. 3, Kel. Cangkiran, Kec. Mijen, Semarang 50216</t>
@@ -1268,10 +1408,26 @@
           <t>DMY009</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Ratna Sari Dewi</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>081234500009</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>ratna.sari@contoh.id</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Tarantang No. 15, Kel. Tarantang, Kec. Lubuk Kilangan, Padang 25151</t>
+        </is>
+      </c>
       <c r="F18" s="5" t="n">
         <v>0</v>
       </c>
@@ -1281,7 +1437,9 @@
       <c r="H18" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I18" s="5" t="n"/>
+      <c r="I18" s="6" t="n">
+        <v>46036</v>
+      </c>
       <c r="J18" s="5" t="n"/>
       <c r="K18" s="5" t="inlineStr">
         <is>
@@ -1305,10 +1463,26 @@
           <t>DMY009</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Ratna Sari Dewi</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>081234500009</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>ratna.sari@contoh.id</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Jl. Tarantang No. 15, Kel. Tarantang, Kec. Lubuk Kilangan, Padang 25151</t>
+        </is>
+      </c>
       <c r="F19" s="5" t="n">
         <v>0</v>
       </c>
@@ -1318,7 +1492,9 @@
       <c r="H19" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="I19" s="5" t="n"/>
+      <c r="I19" s="6" t="n">
+        <v>46036</v>
+      </c>
       <c r="J19" s="5" t="n"/>
       <c r="K19" s="5" t="inlineStr">
         <is>
@@ -1352,7 +1528,11 @@
           <t>081234500010</t>
         </is>
       </c>
-      <c r="D20" s="5" t="n"/>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>hijrah.barokah@contoh.id</t>
+        </is>
+      </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Jl. 35 Ilir No. 27, Kel. 35 Ilir, Kec. Ilir Barat II, Palembang 30144</t>
@@ -1393,10 +1573,26 @@
           <t>DMY010</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Komunitas Hijrah Barokah</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>081234500010</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>hijrah.barokah@contoh.id</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Jl. 35 Ilir No. 27, Kel. 35 Ilir, Kec. Ilir Barat II, Palembang 30144</t>
+        </is>
+      </c>
       <c r="F21" s="5" t="n">
         <v>3</v>
       </c>
@@ -1406,7 +1602,9 @@
       <c r="H21" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="5" t="n"/>
+      <c r="I21" s="6" t="n">
+        <v>46037</v>
+      </c>
       <c r="J21" s="5" t="n"/>
       <c r="K21" s="5" t="inlineStr">
         <is>
@@ -1430,10 +1628,26 @@
           <t>DMY010</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Komunitas Hijrah Barokah</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>081234500010</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>hijrah.barokah@contoh.id</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Jl. 35 Ilir No. 27, Kel. 35 Ilir, Kec. Ilir Barat II, Palembang 30144</t>
+        </is>
+      </c>
       <c r="F22" s="5" t="n">
         <v>0</v>
       </c>
@@ -1443,7 +1657,9 @@
       <c r="H22" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I22" s="5" t="n"/>
+      <c r="I22" s="6" t="n">
+        <v>46037</v>
+      </c>
       <c r="J22" s="5" t="n"/>
       <c r="K22" s="5" t="inlineStr">
         <is>
@@ -1467,10 +1683,26 @@
           <t>DMY010</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Komunitas Hijrah Barokah</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>081234500010</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>hijrah.barokah@contoh.id</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Jl. 35 Ilir No. 27, Kel. 35 Ilir, Kec. Ilir Barat II, Palembang 30144</t>
+        </is>
+      </c>
       <c r="F23" s="5" t="n">
         <v>0</v>
       </c>
@@ -1480,7 +1712,9 @@
       <c r="H23" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="I23" s="5" t="n"/>
+      <c r="I23" s="6" t="n">
+        <v>46037</v>
+      </c>
       <c r="J23" s="5" t="n"/>
       <c r="K23" s="5" t="n"/>
       <c r="L23" s="5" t="inlineStr">

</xml_diff>